<commit_message>
WIP: Switch to TF.js inference, convert Keras 3 topology, add model assets
</commit_message>
<xml_diff>
--- a/Concrete_Crack/Concrete_Crack_DataSource.xlsx
+++ b/Concrete_Crack/Concrete_Crack_DataSource.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Shen\UM_class\SeniorDesign\2026\MobileCrack\Concrete_Crack\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rehab Jadallah\Desktop\SD_Crack_Classification\Concrete_Crack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1034E99-B3FF-4812-8598-553C0E931AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDDA13DF-4DD4-465E-B9EF-64FB5FFF8D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5268" yWindow="372" windowWidth="17724" windowHeight="11364" xr2:uid="{13068FA9-3BE6-4B23-964F-2C325702FB95}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{13068FA9-3BE6-4B23-964F-2C325702FB95}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="106">
   <si>
     <t>File Name</t>
   </si>
@@ -348,13 +348,19 @@
   </si>
   <si>
     <t>Lift Right Concrete</t>
+  </si>
+  <si>
+    <t>https://digitalcommons.usu.edu/all_datasets/48/?</t>
+  </si>
+  <si>
+    <t>USU Campus Concrete</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -366,6 +372,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -388,14 +402,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -708,7 +725,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{962A0094-52C7-46EA-A416-89F71C2E54F3}">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1474,8 +1491,19 @@
         <v>102</v>
       </c>
     </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B71" t="s">
+        <v>105</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C71" r:id="rId1" xr:uid="{56100190-5657-4A8F-9623-9B7553E57AEB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>